<commit_message>
BRD-03 sign-off set: Sales Organisation tree table, Package Version validation and rule parameters of the incentive criteria in the screen specifications, FRS, messages and test cases; screenshots retaken (sales organisation tree, actions menu and refused deactivation, package version header and validation, new incentive criterion, walkthrough steps A-16 and A-17); FRS, sign-off workbook, guide deck and test plan v2.0 rebuilt; allow-list entries of the former rule parameter texts removed from the pack check
</commit_message>
<xml_diff>
--- a/docs/deliverables/out/Drop-0_Setup_and_Data_Migration/BRD-03_Product_Maintenance/04_BIBS_TestPlan_BRD-03_Product_Maintenance_v2.0.xlsx
+++ b/docs/deliverables/out/Drop-0_Setup_and_Data_Migration/BRD-03_Product_Maintenance/04_BIBS_TestPlan_BRD-03_Product_Maintenance_v2.0.xlsx
@@ -10343,7 +10343,7 @@
       </c>
       <c r="D134" s="12" t="inlineStr">
         <is>
-          <t>A criterion on an inactive product, without products or value, with invalid rule parameters or an overlapping period cannot be saved.</t>
+          <t>A criterion on an inactive product, without products or value, with a rule parameter without a valid value or an overlapping period cannot be saved.</t>
         </is>
       </c>
       <c r="E134" s="12" t="inlineStr">
@@ -27270,7 +27270,7 @@
       </c>
       <c r="E218" s="12" t="inlineStr">
         <is>
-          <t>Rule parameters not in the format of the example</t>
+          <t>Rule parameter value that is not a number</t>
         </is>
       </c>
       <c r="F218" s="12" t="inlineStr">
@@ -27300,13 +27300,13 @@
       </c>
       <c r="K218" s="12" t="inlineStr">
         <is>
-          <t>1. Value basis Rule, rule parameters "{minimumPremium 5000"; save.</t>
+          <t>1. Value basis Rule; Add Parameter, parameter Minimum Gross Premium, value "five thousand"; save.</t>
         </is>
       </c>
       <c r="L218" s="12" t="inlineStr">
         <is>
-          <t>Not saved.
-Message "The rule parameters must be valid JSON" (INCENTIVE_RULE_PARAMS_INVALID).</t>
+          <t>Not saved; the message is under the value.
+Message "Minimum Gross Premium must be a number" (INCENTIVE_RULE_PARAMS_INVALID).</t>
         </is>
       </c>
       <c r="M218" s="12" t="inlineStr">
@@ -28997,7 +28997,7 @@
       <c r="L240" s="12" t="inlineStr">
         <is>
           <t>The screen matches SCR-PM-13 Package Version of the FRS.
-Fields in this order: 1 Product / Version (Reference chip, mandatory -); 2 Version status pill (Pill, mandatory -); 3 Request tag (Tag, mandatory -); 4 Effective / Package End / Rate % / Set Up By / ManCom Ref. (Fact, mandatory -); 5 Package Rate % (Number, mandatory Cond.: or a rate for every insurer); 6 Minimum Premium (Number, mandatory Y); 7 Commission % (Number, mandatory Y); 8 Package TSI Limit (Number, mandatory N); 9 Effective From (Date, mandatory Y); 10 Package Start (Date, mandatory N); 11 Package End (Date, mandatory N); 12 Anniversary (Date, mandatory N); 13 Change Summary (Text, mandatory N); 14 ManCom Sign-off Reference (Text, mandatory N); 15 Computation Basis (Text, mandatory N); 16 Coverage (Column, mandatory Y (at least one included)); 17 Included / Optional (Check box, mandatory N); 18 Limit / Deductible (Number, mandatory N); 19 Add coverage (Drop-down, mandatory N); 20 Insurer (Column, mandatory N); 21 Role (Drop-down, mandatory Y); 22 Share % (Number, mandatory Cond.: lead and participants); 23 Rate % (Number, mandatory Cond.: when there is no package rate); 24 Minimum Premium (Number, mandatory N); 25 Add insurer (Drop-down, mandatory N); 26 Insurer / Coverage (Column, mandatory Y (every pair)); 27 Covered (Check box, mandatory N); 28 Limit / Deductible / Deductible Wording (Number / Text, mandatory N); 29 Clauses (Multi-select, mandatory N); 30 Hierarchy complete: cover type and basic coverage / Every panel insurer has terms for each included coverage / Rates and minimum premiums match the signed-off terms / Dates and package term are correct / Test premium reviewed (Check box, mandatory Y (all five)); 31 Validated by, date and test premium (Detail, mandatory -); 32 Return reason / Comment (Drop-down / Text, mandatory Y (reason)).
+Fields in this order: 1 Product / Version (Reference chip, mandatory -); 2 Version status pill (Pill, mandatory -); 3 Effective / Package End / Rate % / Set Up By / ManCom Ref. (Fact, mandatory -); 4 Package Request (Fact, mandatory -); 5 Package Rate % (Number, mandatory Cond.: or a rate for every insurer); 6 Minimum Premium (Number, mandatory Y); 7 Commission % (Number, mandatory Y); 8 Package TSI Limit (Number, mandatory N); 9 Effective From (Date, mandatory Y); 10 Package Start (Date, mandatory N); 11 Package End (Date, mandatory N); 12 Anniversary (Date, mandatory N); 13 Change Summary (Text, mandatory N); 14 ManCom Sign-off Reference (Text, mandatory N); 15 Computation Basis (Text, mandatory N); 16 Coverage (Column, mandatory Y (at least one included)); 17 Included / Optional (Check box, mandatory N); 18 Limit / Deductible (Number, mandatory N); 19 Add coverage (Drop-down, mandatory N); 20 Insurer (Column, mandatory N); 21 Role (Drop-down, mandatory Y); 22 Share % (Number, mandatory Cond.: lead and participants); 23 Rate % (Number, mandatory Cond.: when there is no package rate); 24 Minimum Premium (Number, mandatory N); 25 Add insurer (Drop-down, mandatory N); 26 Insurer / Coverage (Column, mandatory Y (every pair)); 27 Covered (Check box, mandatory N); 28 Limit / Deductible / Deductible Wording (Number / Text, mandatory N); 29 Clauses (Multi-select, mandatory N); 30 Hierarchy complete: cover type and basic coverage / Every panel insurer has terms for each included coverage / Rates and minimum premiums match the signed-off terms / Dates and package term are correct / Test premium reviewed (Check box, mandatory Y (all five)); 31 Result / Validated By / Validated On / Test Premium / Return Reason (Fact, mandatory -); 32 # / Check / Result / Details (Table, mandatory -); 33 Return reason / Comment (Drop-down / Text, mandatory Y (reason)).
 Actions: Save Draft; Submit for Validation; Validate and Release; Return to MBS.
 The message of the field table is shown word for word and nothing is saved.</t>
         </is>
@@ -29234,7 +29234,7 @@
       <c r="L243" s="12" t="inlineStr">
         <is>
           <t>The screen matches SCR-PM-16 Incentive Criteria of the FRS.
-Fields in this order: 1 Current / Pending Authorization / History (Tab, mandatory -); 2 Search Criterion or Product (Text, mandatory N); 3 Code / Name / Type / Value / Products / From / Until / Status (Column, mandatory -); 4 Code (Text, mandatory Y); 5 Name (Text, mandatory Y); 6 Incentive type (Drop-down, mandatory Y); 7 Value basis (Drop-down, mandatory Y); 8 Value (Number, mandatory Cond.: rate or fixed amount); 9 Effective from (Date, mandatory Y); 10 Effective to (Date, mandatory N); 11 Rule parameters (JSON) (Text, mandatory N); 12 Description (Text, mandatory N); 13 Products matrix (Drop-down and rows, mandatory Y (at least one)).
+Fields in this order: 1 Current / Pending Authorization / History (Tab, mandatory -); 2 Search Criterion or Product (Text, mandatory N); 3 Code / Name / Type / Value / Products / From / Until / Status (Column, mandatory -); 4 Code (Text, mandatory Y); 5 Name (Text, mandatory Y); 6 Incentive type (Drop-down, mandatory Y); 7 Value basis (Drop-down, mandatory Y); 8 Value (Number, mandatory Cond.: rate or fixed amount); 9 Effective from (Date, mandatory Y); 10 Effective to (Date, mandatory N); 11 Rule Parameters (Rows: parameter and value, mandatory N (a value per row)); 12 Description (Text, mandatory N); 13 Products matrix (Drop-down and rows, mandatory Y (at least one)).
 Actions: New Criterion; Open a row; Authorize; Deactivate.
 The message of the field table is shown word for word and nothing is saved.</t>
         </is>
@@ -29542,8 +29542,8 @@
       <c r="L247" s="12" t="inlineStr">
         <is>
           <t>The screen matches SCR-PM-20 Sales Organisation of the FRS.
-Fields in this order: 1 Unit line (Tree, mandatory -); 2 Account officer line (Tree, mandatory -); 3 Level (Drop-down, mandatory Y); 4 Code / Name (Text, mandatory Y); 5 Cost center (Text, mandatory N); 6 Parent (Drop-down, mandatory Cond.: department and team); 7 Team (Drop-down, mandatory Y); 8 User name (Text, mandatory Y).
-Actions: New Unit; Assign Officer; Authorize / Deactivate.
+Fields in this order: 1 Search unit code, name or officer (Text, mandatory N); 2 Expand All / Collapse All (Button, mandatory -); 3 Show Inactive (Check box, mandatory N); 4 Summary (Text, mandatory -); 5 Unit (Column, mandatory -); 6 Level (Column, mandatory -); 7 Cost Center (Column, mandatory -); 8 Account Officers (Column, mandatory -); 9 Assigned Since (Column, mandatory -); 10 Status (Pill, mandatory -); 11 Actions (Menu, mandatory -); 12 Level (Drop-down, mandatory Y); 13 Code / Name (Text, mandatory Y); 14 Cost Center (Text, mandatory N); 15 Parent (Drop-down, mandatory Cond.: department and team); 16 Code, Name, Level, Parent Unit, Cost Center, Unit Head, Sub-units, Account Officers, Status, Status Reason, Created, Last Changed, Authorized (Detail, mandatory -); 17 Team (Drop-down, mandatory Y); 18 Account Officer (Drop-down, mandatory Y); 19 Reason (Text, mandatory Y).
+Actions: New Unit; Assign Officer; View / Edit; Add Department / Add Team; Assign Officer (row); Authorize; Deactivate; Reactivate; Reassign / Assign to a Team; Remove from Team; Export to Excel.
 The message of the field table is shown word for word and nothing is saved.</t>
         </is>
       </c>
@@ -30629,21 +30629,21 @@
 MSG-PM-139: "Enter the minimum premium"
 MSG-PM-140: "Enter the package rate or a rate for every insurer"
 MSG-PM-141: "Include at least one coverage"
-MSG-PM-144: "The effective date cannot be before today"
-MSG-PM-145: "The package end date must be after the effective date"
-MSG-PM-146: "The package version is validated and released for use."
-MSG-PM-149: "A package version is validated by someone other than its maker and submitter" (MAKER_CHECKER_VIOLATION)
-MSG-PM-150: "Package version not found: &lt;version no&gt;" (NOT_FOUND)
-MSG-PM-151: "Enter the effective date" (PACKAGE_DATES_INVALID)
-MSG-PM-152: "The effective date cannot be before today" (PACKAGE_DATES_INVALID)
-MSG-PM-153: "The effective date must be after the start of version &lt;version no&gt;" (PACKAGE_DATES_INVALID)
-MSG-PM-154: "The package end date must be after the effective date" (PACKAGE_DATES_INVALID)
-MSG-PM-155: "The package needs its cover type and at least one included basic coverage" (PACKAGE_HIERARCHY_INCOMPLETE)
-MSG-PM-156: "Insurer &lt;insurer code&gt; has no terms for coverage &lt;coverage&gt;" (PACKAGE_INSURER_TERMS_MISSING)
-MSG-PM-157: "Enter the package rate or a rate for every insurer" (PACKAGE_RATE_MISSING)
-MSG-PM-158: "The co-insurance shares must add up to 100%" (PACKAGE_SHARES_INVALID)
-MSG-PM-159: "Enter the reason of the return" (REASON_REQUIRED)
-MSG-PM-160: "Version &lt;version no&gt; is &lt;status&gt;" (VERSION_NOT_FOR_VALIDATION)</t>
+MSG-PM-145: "The effective date cannot be before today"
+MSG-PM-146: "The package end date must be after the effective date"
+MSG-PM-147: "The package version is validated and released for use."
+MSG-PM-150: "A package version is validated by someone other than its maker and submitter" (MAKER_CHECKER_VIOLATION)
+MSG-PM-151: "Package version not found: &lt;version no&gt;" (NOT_FOUND)
+MSG-PM-152: "Enter the effective date" (PACKAGE_DATES_INVALID)
+MSG-PM-153: "The effective date cannot be before today" (PACKAGE_DATES_INVALID)
+MSG-PM-154: "The effective date must be after the start of version &lt;version no&gt;" (PACKAGE_DATES_INVALID)
+MSG-PM-155: "The package end date must be after the effective date" (PACKAGE_DATES_INVALID)
+MSG-PM-156: "The package needs its cover type and at least one included basic coverage" (PACKAGE_HIERARCHY_INCOMPLETE)
+MSG-PM-157: "Insurer &lt;insurer code&gt; has no terms for coverage &lt;coverage&gt;" (PACKAGE_INSURER_TERMS_MISSING)
+MSG-PM-158: "Enter the package rate or a rate for every insurer" (PACKAGE_RATE_MISSING)
+MSG-PM-159: "The co-insurance shares must add up to 100%" (PACKAGE_SHARES_INVALID)
+MSG-PM-160: "Enter the reason of the return" (REASON_REQUIRED)
+MSG-PM-161: "Version &lt;version no&gt; is &lt;status&gt;" (VERSION_NOT_FOR_VALIDATION)</t>
         </is>
       </c>
       <c r="M260" s="12" t="inlineStr">
@@ -30718,17 +30718,17 @@
       <c r="L261" s="12" t="inlineStr">
         <is>
           <t>Each message is shown word for word, with its code as the Reference for a server message, and nothing is saved:
-MSG-PM-163: "Enter the effective date"
-MSG-PM-164: "Enter the name"
-MSG-PM-165: "Enter the title"
-MSG-PM-166: "Enter the wording"
-MSG-PM-168: "Select the kind"
-MSG-PM-169: "Select the product line"
-MSG-PM-171: "The end is before the start"
-MSG-PM-172: "Use A-Z, 0-9 and _"
-MSG-PM-173: "&lt;label&gt; already exists: &lt;key&gt;" (DUPLICATE)
-MSG-PM-174: "&lt;label&gt; not found: &lt;code&gt;" (NOT_FOUND)
-MSG-PM-175: "&lt;label&gt; not found: &lt;id&gt;" (NOT_FOUND)</t>
+MSG-PM-164: "Enter the effective date"
+MSG-PM-165: "Enter the name"
+MSG-PM-166: "Enter the title"
+MSG-PM-167: "Enter the wording"
+MSG-PM-169: "Select the kind"
+MSG-PM-170: "Select the product line"
+MSG-PM-172: "The end is before the start"
+MSG-PM-173: "Use A-Z, 0-9 and _"
+MSG-PM-174: "&lt;label&gt; already exists: &lt;key&gt;" (DUPLICATE)
+MSG-PM-175: "&lt;label&gt; not found: &lt;code&gt;" (NOT_FOUND)
+MSG-PM-176: "&lt;label&gt; not found: &lt;id&gt;" (NOT_FOUND)</t>
         </is>
       </c>
       <c r="M261" s="12" t="inlineStr">
@@ -30803,24 +30803,25 @@
       <c r="L262" s="12" t="inlineStr">
         <is>
           <t>Each message is shown word for word, with its code as the Reference for a server message, and nothing is saved:
-MSG-PM-178: "Enter the name"
-MSG-PM-179: "Enter the start date"
-MSG-PM-180: "Enter the value"
-MSG-PM-181: "Enter valid JSON, e.g. {"minimumPremium": 5000}"
-MSG-PM-182: "Select at least one product of the matrix"
-MSG-PM-183: "Select the type"
-MSG-PM-184: "The change must start after &lt;active from&gt;"
-MSG-PM-185: "The end is before the start"
-MSG-PM-186: "Use A-Z, 0-9, _ and -"
-MSG-PM-187: "An active criterion is changed by amending it (successor)" (INCENTIVE_ACTIVE_LOCKED)
-MSG-PM-188: "Only an active criterion is amended; change the pending row" (INCENTIVE_NOT_ACTIVE)
-MSG-PM-189: "The amendment must start after &lt;effective from&gt;" (INCENTIVE_PERIOD_INVALID)
-MSG-PM-190: "Criterion &lt;code&gt; already covers part of this period" (INCENTIVE_PERIOD_OVERLAP)
-MSG-PM-191: "Select at least one product of the products matrix" (INCENTIVE_PRODUCTS_REQUIRED)
-MSG-PM-192: "Product &lt;product code&gt; is not an active product of the matrix" (INCENTIVE_PRODUCT_NOT_ACTIVE)
-MSG-PM-193: "The rule parameters must be valid JSON" (INCENTIVE_RULE_PARAMS_INVALID)
-MSG-PM-194: "Enter the value of the incentive criterion" (INCENTIVE_VALUE_REQUIRED)
-MSG-PM-195: "&lt;label&gt; not found: &lt;id&gt;" (NOT_FOUND)</t>
+MSG-PM-179: "Enter a value for each parameter"
+MSG-PM-180: "Enter the name"
+MSG-PM-181: "Enter the start date"
+MSG-PM-182: "Enter the value"
+MSG-PM-183: "Select at least one product of the matrix"
+MSG-PM-184: "Select the parameter"
+MSG-PM-185: "Select the type"
+MSG-PM-186: "The change must start after &lt;active from&gt;"
+MSG-PM-187: "The end is before the start"
+MSG-PM-188: "Use A-Z, 0-9, _ and -"
+MSG-PM-189: "An active criterion is changed by amending it (successor)" (INCENTIVE_ACTIVE_LOCKED)
+MSG-PM-190: "Only an active criterion is amended; change the pending row" (INCENTIVE_NOT_ACTIVE)
+MSG-PM-191: "The amendment must start after &lt;effective from&gt;" (INCENTIVE_PERIOD_INVALID)
+MSG-PM-192: "Criterion &lt;code&gt; already covers part of this period" (INCENTIVE_PERIOD_OVERLAP)
+MSG-PM-193: "Select at least one product of the products matrix" (INCENTIVE_PRODUCTS_REQUIRED)
+MSG-PM-194: "Product &lt;product code&gt; is not an active product of the matrix" (INCENTIVE_PRODUCT_NOT_ACTIVE)
+MSG-PM-195: "Enter the rule parameters as parameter and value rows" (INCENTIVE_RULE_PARAMS_INVALID)
+MSG-PM-196: "Enter the value of the incentive criterion" (INCENTIVE_VALUE_REQUIRED)
+MSG-PM-197: "&lt;label&gt; not found: &lt;id&gt;" (NOT_FOUND)</t>
         </is>
       </c>
       <c r="M262" s="12" t="inlineStr">
@@ -30895,17 +30896,17 @@
       <c r="L263" s="12" t="inlineStr">
         <is>
           <t>Each message is shown word for word, with its code as the Reference for a server message, and nothing is saved:
-MSG-PM-198: "Default credit days must be between 0 and 365" (CREDIT_DAYS_INVALID)
-MSG-PM-199: "&lt;label&gt; already exists: &lt;key&gt;" (DUPLICATE)
-MSG-PM-200: "Branch &lt;branch code&gt; is not authorized or inactive" (INSURER_BRANCH_NOT_ACTIVE)
-MSG-PM-201: "Insurer &lt;party code&gt; has no branch &lt;branch code&gt;" (INSURER_BRANCH_UNKNOWN)
-MSG-PM-202: "Insurer &lt;party code&gt; is not authorized or is inactive" (INSURER_NOT_ACTIVE)
-MSG-PM-203: "&lt;label&gt; not found: &lt;branch id&gt;" (NOT_FOUND)
-MSG-PM-204: "&lt;label&gt; not found: &lt;id&gt;" (NOT_FOUND)
-MSG-PM-205: "&lt;label&gt; not found: &lt;party code&gt;" (NOT_FOUND)
-MSG-PM-206: "Party &lt;party code&gt; exists and is not an insurer" (PARTY_NOT_INSURER)
-MSG-PM-207: "Only e-mail placement is available; choose the e-mail placement channel" (PLACEMENT_CHANNEL_PARKED)
-MSG-PM-208: "The LGT rate must be between 0 and 100 %" (RATE_INVALID)</t>
+MSG-PM-200: "Default credit days must be between 0 and 365" (CREDIT_DAYS_INVALID)
+MSG-PM-201: "&lt;label&gt; already exists: &lt;key&gt;" (DUPLICATE)
+MSG-PM-202: "Branch &lt;branch code&gt; is not authorized or inactive" (INSURER_BRANCH_NOT_ACTIVE)
+MSG-PM-203: "Insurer &lt;party code&gt; has no branch &lt;branch code&gt;" (INSURER_BRANCH_UNKNOWN)
+MSG-PM-204: "Insurer &lt;party code&gt; is not authorized or is inactive" (INSURER_NOT_ACTIVE)
+MSG-PM-205: "&lt;label&gt; not found: &lt;branch id&gt;" (NOT_FOUND)
+MSG-PM-206: "&lt;label&gt; not found: &lt;id&gt;" (NOT_FOUND)
+MSG-PM-207: "&lt;label&gt; not found: &lt;party code&gt;" (NOT_FOUND)
+MSG-PM-208: "Party &lt;party code&gt; exists and is not an insurer" (PARTY_NOT_INSURER)
+MSG-PM-209: "Only e-mail placement is available; choose the e-mail placement channel" (PLACEMENT_CHANNEL_PARKED)
+MSG-PM-210: "The LGT rate must be between 0 and 100 %" (RATE_INVALID)</t>
         </is>
       </c>
       <c r="M263" s="12" t="inlineStr">
@@ -30980,13 +30981,13 @@
       <c r="L264" s="12" t="inlineStr">
         <is>
           <t>Each message is shown word for word, with its code as the Reference for a server message, and nothing is saved:
-MSG-PM-212: "Enter the effective-from date" (EFFECTIVE_FROM_REQUIRED)
-MSG-PM-213: "The effective-to date is before the effective-from date" (EFFECTIVITY_INVALID)
-MSG-PM-214: "The limit must be greater than zero" (LIMIT_INVALID)
-MSG-PM-215: "The premium cannot be negative" (LIMIT_PREMIUM_INVALID)
-MSG-PM-216: "&lt;label&gt; not found: &lt;id&gt;" (NOT_FOUND)
-MSG-PM-217: "&lt;label&gt; must be a percentage between 0 and 100" (RATE_INVALID)
-MSG-PM-218: "Months covered must be between 1 and 12" (SHORT_PERIOD_MONTHS_INVALID)</t>
+MSG-PM-214: "Enter the effective-from date" (EFFECTIVE_FROM_REQUIRED)
+MSG-PM-215: "The effective-to date is before the effective-from date" (EFFECTIVITY_INVALID)
+MSG-PM-216: "The limit must be greater than zero" (LIMIT_INVALID)
+MSG-PM-217: "The premium cannot be negative" (LIMIT_PREMIUM_INVALID)
+MSG-PM-218: "&lt;label&gt; not found: &lt;id&gt;" (NOT_FOUND)
+MSG-PM-219: "&lt;label&gt; must be a percentage between 0 and 100" (RATE_INVALID)
+MSG-PM-220: "Months covered must be between 1 and 12" (SHORT_PERIOD_MONTHS_INVALID)</t>
         </is>
       </c>
       <c r="M264" s="12" t="inlineStr">
@@ -31053,13 +31054,19 @@
       <c r="L265" s="12" t="inlineStr">
         <is>
           <t>Each message is shown word for word, with its code as the Reference for a server message, and nothing is saved:
-MSG-PM-220: "&lt;label&gt; already exists: &lt;key&gt;" (DUPLICATE)
-MSG-PM-221: "&lt;label&gt; not found: &lt;id&gt;" (NOT_FOUND)
-MSG-PM-222: "&lt;label&gt; not found: &lt;unit code&gt;" (NOT_FOUND)
-MSG-PM-223: "A &lt;level&gt; must belong to a &lt;parent level&gt;" (SALES_PARENT_INVALID)
-MSG-PM-224: "Unknown team &lt;team code&gt;" (SALES_TEAM_UNKNOWN)
-MSG-PM-225: "Unknown user &lt;head&gt;" (USER_UNKNOWN)
-MSG-PM-226: "Unknown user &lt;username&gt;" (USER_UNKNOWN)</t>
+MSG-PM-228: "&lt;label&gt; already exists: &lt;key&gt;" (DUPLICATE)
+MSG-PM-229: "&lt;label&gt; not found: &lt;id&gt;" (NOT_FOUND)
+MSG-PM-230: "&lt;label&gt; not found: &lt;unit code&gt;" (NOT_FOUND)
+MSG-PM-231: "Enter the reason" (REASON_REQUIRED)
+MSG-PM-232: "&lt;&gt; is already removed from the team" (SALES_OFFICER_INACTIVE)
+MSG-PM-233: "A &lt;level&gt; must belong to an active &lt;parent level&gt;" (SALES_PARENT_INVALID)
+MSG-PM-234: "Reactivate &lt;parent code&gt; before &lt;code&gt;" (SALES_PARENT_INVALID)
+MSG-PM-235: "Team &lt;team code&gt; is unknown or inactive" (SALES_TEAM_UNKNOWN)
+MSG-PM-236: "Unit &lt;code&gt; is already inactive" (SALES_UNIT_INACTIVE)
+MSG-PM-237: "&lt;code&gt; still has &lt;open&gt;: deactivate or move them before deactivating the unit" (SALES_UNIT_IN_USE)
+MSG-PM-238: "Unit &lt;code&gt; is not inactive" (SALES_UNIT_NOT_INACTIVE)
+MSG-PM-239: "Unknown user &lt;head&gt;" (USER_UNKNOWN)
+MSG-PM-240: "Unknown user &lt;username&gt;" (USER_UNKNOWN)</t>
         </is>
       </c>
       <c r="M265" s="12" t="inlineStr">
@@ -31134,18 +31141,18 @@
       <c r="L266" s="12" t="inlineStr">
         <is>
           <t>Each message is shown word for word, with its code as the Reference for a server message, and nothing is saved:
-MSG-PM-227: "Insurer &lt;insurer code&gt; is not on the panel of &lt;product code&gt; version &lt;version no&gt;" (INSURER_NOT_ON_PACKAGE)
-MSG-PM-228: "&lt;coverage&gt; limit &lt;to plain string&gt; is not in the limit table" (MOTOR_LIMIT_UNKNOWN)
-MSG-PM-229: "Package &lt;code&gt; expired and has no current version" (PRODUCT_NOT_SELLABLE)
-MSG-PM-230: "Package &lt;code&gt; has no released version in force" (PRODUCT_NOT_SELLABLE)
-MSG-PM-231: "Package &lt;code&gt; is &lt;lifecycle status&gt;: it is locked for new business" (PRODUCT_NOT_SELLABLE)
-MSG-PM-232: "Enter at least one item to rate" (RATING_NO_ITEMS)
-MSG-PM-233: "The motor OD/Theft coverage factor is not set up" (RATING_OD_FACTOR_MISSING)
-MSG-PM-234: "The period end must be after the period start" (RATING_PERIOD_INVALID)
-MSG-PM-235: "Enter the premium rate of &lt;item&gt;" (RATING_RATE_REQUIRED)
-MSG-PM-236: "No short-period percentage applies to this period" (RATING_SHORT_PERIOD_INVALID)
-MSG-PM-237: "Enter a sum insured of zero or more for every item" (RATING_SUM_INSURED_INVALID)
-MSG-PM-238: "No short-period rate is set up for &lt;months&gt; month(s)" (SHORT_PERIOD_RATE_MISSING)</t>
+MSG-PM-241: "Insurer &lt;insurer code&gt; is not on the panel of &lt;product code&gt; version &lt;version no&gt;" (INSURER_NOT_ON_PACKAGE)
+MSG-PM-242: "&lt;coverage&gt; limit &lt;to plain string&gt; is not in the limit table" (MOTOR_LIMIT_UNKNOWN)
+MSG-PM-243: "Package &lt;code&gt; expired and has no current version" (PRODUCT_NOT_SELLABLE)
+MSG-PM-244: "Package &lt;code&gt; has no released version in force" (PRODUCT_NOT_SELLABLE)
+MSG-PM-245: "Package &lt;code&gt; is &lt;lifecycle status&gt;: it is locked for new business" (PRODUCT_NOT_SELLABLE)
+MSG-PM-246: "Enter at least one item to rate" (RATING_NO_ITEMS)
+MSG-PM-247: "The motor OD/Theft coverage factor is not set up" (RATING_OD_FACTOR_MISSING)
+MSG-PM-248: "The period end must be after the period start" (RATING_PERIOD_INVALID)
+MSG-PM-249: "Enter the premium rate of &lt;item&gt;" (RATING_RATE_REQUIRED)
+MSG-PM-250: "No short-period percentage applies to this period" (RATING_SHORT_PERIOD_INVALID)
+MSG-PM-251: "Enter a sum insured of zero or more for every item" (RATING_SUM_INSURED_INVALID)
+MSG-PM-252: "No short-period rate is set up for &lt;months&gt; month(s)" (SHORT_PERIOD_RATE_MISSING)</t>
         </is>
       </c>
       <c r="M266" s="12" t="inlineStr">
@@ -31220,14 +31227,14 @@
       <c r="L267" s="12" t="inlineStr">
         <is>
           <t>Each message is shown word for word, with its code as the Reference for a server message, and nothing is saved:
-MSG-PM-240: "A rate exception is decided by someone other than its requester" (MAKER_CHECKER_VIOLATION)
-MSG-PM-241: "&lt;label&gt; not found: &lt;reference&gt;" (NOT_FOUND)
-MSG-PM-242: "Only package rate schemes need an exception" (PRODUCT_NOT_PACKAGED)
-MSG-PM-243: "Enter the version or the rate the exception is for" (RATE_EXCEPTION_INCOMPLETE)
-MSG-PM-244: "The validity date cannot be in the past" (RATE_EXCEPTION_VALIDITY_PAST)
-MSG-PM-245: "Package &lt;product code&gt; is priced on the current rate scheme: &lt;what&gt; needs an approved rate exception" (RATE_SCHEME_NOT_CURRENT)
-MSG-PM-246: "Rate exception &lt;reference&gt; does not approve &lt;what&gt; for &lt;product code&gt;" (RATE_SCHEME_NOT_CURRENT)
-MSG-PM-247: "Rate exception &lt;reference no&gt; is already decided" (RECORD_NOT_PENDING)</t>
+MSG-PM-254: "A rate exception is decided by someone other than its requester" (MAKER_CHECKER_VIOLATION)
+MSG-PM-255: "&lt;label&gt; not found: &lt;reference&gt;" (NOT_FOUND)
+MSG-PM-256: "Only package rate schemes need an exception" (PRODUCT_NOT_PACKAGED)
+MSG-PM-257: "Enter the version or the rate the exception is for" (RATE_EXCEPTION_INCOMPLETE)
+MSG-PM-258: "The validity date cannot be in the past" (RATE_EXCEPTION_VALIDITY_PAST)
+MSG-PM-259: "Package &lt;product code&gt; is priced on the current rate scheme: &lt;what&gt; needs an approved rate exception" (RATE_SCHEME_NOT_CURRENT)
+MSG-PM-260: "Rate exception &lt;reference&gt; does not approve &lt;what&gt; for &lt;product code&gt;" (RATE_SCHEME_NOT_CURRENT)
+MSG-PM-261: "Rate exception &lt;reference no&gt; is already decided" (RECORD_NOT_PENDING)</t>
         </is>
       </c>
       <c r="M267" s="12" t="inlineStr">
@@ -31290,7 +31297,7 @@
       <c r="L268" s="12" t="inlineStr">
         <is>
           <t>Each message is shown word for word, with its code as the Reference for a server message, and nothing is saved:
-MSG-PM-248: "&lt;label&gt; not found: &lt;id&gt;" (NOT_FOUND)</t>
+MSG-PM-262: "&lt;label&gt; not found: &lt;id&gt;" (NOT_FOUND)</t>
         </is>
       </c>
       <c r="M268" s="12" t="inlineStr">
@@ -31353,13 +31360,13 @@
       <c r="L269" s="12" t="inlineStr">
         <is>
           <t>Each message is shown word for word, with its code as the Reference for a server message, and nothing is saved:
-MSG-PM-249: "You are not permitted to perform this action" (ACCESS_DENIED)
-MSG-PM-250: "The record was changed by another user. Please reload and try again." (CONCURRENT_MODIFICATION)
-MSG-PM-252: "The system could not complete the request. Try again; if it continues, contact support with the reference." (INTERNAL_ERROR)
-MSG-PM-254: "Parameter '&lt;name&gt;' has an invalid value" (MALFORMED_REQUEST)
-MSG-PM-255: "Required parameter '&lt;parameter name&gt;' is missing" (MALFORMED_REQUEST)
-MSG-PM-260: "The uploaded file is too large" (UPLOAD_TOO_LARGE)
-MSG-PM-261: "Invalid request" (VALIDATION_FAILED)</t>
+MSG-PM-263: "You are not permitted to perform this action" (ACCESS_DENIED)
+MSG-PM-264: "The record was changed by another user. Please reload and try again." (CONCURRENT_MODIFICATION)
+MSG-PM-266: "The system could not complete the request. Try again; if it continues, contact support with the reference." (INTERNAL_ERROR)
+MSG-PM-268: "Parameter '&lt;name&gt;' has an invalid value" (MALFORMED_REQUEST)
+MSG-PM-269: "Required parameter '&lt;parameter name&gt;' is missing" (MALFORMED_REQUEST)
+MSG-PM-274: "The uploaded file is too large" (UPLOAD_TOO_LARGE)
+MSG-PM-275: "Invalid request" (VALIDATION_FAILED)</t>
         </is>
       </c>
       <c r="M269" s="12" t="inlineStr">
@@ -31422,12 +31429,12 @@
       <c r="L270" s="12" t="inlineStr">
         <is>
           <t>Each message is shown word for word, with its code as the Reference for a server message, and nothing is saved:
-MSG-PM-251: "&lt;label&gt; already exists: &lt;key&gt;" (DUPLICATE)
-MSG-PM-253: "A rate exception is decided by someone other than its requester" (MAKER_CHECKER_VIOLATION)
-MSG-PM-256: "&lt;label&gt; not found: &lt;id&gt;" (NOT_FOUND)
-MSG-PM-257: "Product &lt;code&gt; was not created by the migration" (PRODUCT_NOT_MIGRATED)
-MSG-PM-258: "Enter the reason for the rejection" (RATE_EXCEPTION_REASON_REQUIRED)
-MSG-PM-259: "Rate exception &lt;reference&gt; is already decided" (RECORD_NOT_PENDING)</t>
+MSG-PM-265: "&lt;label&gt; already exists: &lt;key&gt;" (DUPLICATE)
+MSG-PM-267: "A rate exception is decided by someone other than its requester" (MAKER_CHECKER_VIOLATION)
+MSG-PM-270: "&lt;label&gt; not found: &lt;id&gt;" (NOT_FOUND)
+MSG-PM-271: "Product &lt;code&gt; was not created by the migration" (PRODUCT_NOT_MIGRATED)
+MSG-PM-272: "Enter the reason for the rejection" (RATE_EXCEPTION_REASON_REQUIRED)
+MSG-PM-273: "Rate exception &lt;reference&gt; is already decided" (RECORD_NOT_PENDING)</t>
         </is>
       </c>
       <c r="M270" s="12" t="inlineStr">

</xml_diff>

<commit_message>
Drop 0 sign-off sets BRD-03, BRD-11 and BRD-13 rebuilt on screenshots retaken on a fresh seed stack: issue 2.1 changes CHG-PM-2.1-01 to 05, CHG-UA-2.1-01 to 05 and CHG-DM-2.1-01 to 05 flagged in the UX documents; 00 to 09 of each set, the Drop 0 closure set and the drop indexes rebuilt with both logos; password steps of the BRD-11 walkthrough cropped to the password card; the closure asks for no parameter of the insurer suite and claims the seeded tax codes
</commit_message>
<xml_diff>
--- a/docs/deliverables/out/Drop-0_Setup_and_Data_Migration/BRD-03_Product_Maintenance/04_BIBS_TestPlan_BRD-03_Product_Maintenance_v2.0.xlsx
+++ b/docs/deliverables/out/Drop-0_Setup_and_Data_Migration/BRD-03_Product_Maintenance/04_BIBS_TestPlan_BRD-03_Product_Maintenance_v2.0.xlsx
@@ -11312,8 +11312,8 @@
       </c>
       <c r="L8" s="12" t="inlineStr">
         <is>
-          <t>The last wrong attempt locks the account; the correct password is then refused until the System Administrator unlocks the user in Administration &gt; Users.
-Message "Account is locked. Contact your administrator." (AUTHENTICATION_FAILED).</t>
+          <t>The last wrong attempt locks the account; the correct password is then refused with the same message as a wrong password until the System Administrator unlocks the user in Administration &gt; Users, where the lock shows.
+Message "Invalid user name or password" (AUTHENTICATION_FAILED).</t>
         </is>
       </c>
       <c r="M8" s="12" t="inlineStr">
@@ -28211,7 +28211,7 @@
       <c r="L230" s="12" t="inlineStr">
         <is>
           <t>The screen matches SCR-PM-03 New Package Request and Edit Package Request of the FRS.
-Fields in this order: 1 Request type (Drop-down, mandatory Y); 2 Scope (Drop-down, mandatory Y); 3 Package / programme name (Text, mandatory Y); 4 Client or prospect (Look-up, mandatory Cond.: client-specific package); 5 Product line (Drop-down, mandatory Y); 6 Cover type / subtype (Drop-down, mandatory Cond.: New package); 7 Package product (Drop-down, mandatory Cond.: every type except New package); 8 Reason (Drop-down, mandatory Y); 9 Comment on the reason (Text, mandatory N); 10 Negotiate with the insurers (Check box, mandatory N); 11 Market segments (Check boxes, mandatory N); 12 Heading / Details (Text, mandatory Cond.: sections or coverages before submission); 13 Coverage code (Text, mandatory Cond.: sections or coverages before submission); 14 Included (Check box, mandatory N); 15 Limit (Number, mandatory N); 16 Deductible (Text, mandatory N); 17 Requested rate % (Number, mandatory N); 18 Minimum premium (Number, mandatory N); 19 Commission % (Number, mandatory N); 20 Package TSI limit (Number, mandatory N); 21 Effective from (Date, mandatory N); 22 Package start (Date, mandatory N); 23 Package end (Date, mandatory Cond.: before submission (not for Retire)); 24 Anniversary (Date, mandatory N); 25 Insurer check boxes (Check boxes, mandatory Cond.: at least one when the insurers are approached); 26 Documents panel (Upload, mandatory N).
+Fields in this order: 1 Request type (Drop-down, mandatory Y); 2 Scope (Drop-down, mandatory Y); 3 Package / programme name (Text, mandatory Y); 4 Client or prospect (Look-up, mandatory Cond.: client-specific package); 5 Product line (Drop-down, mandatory Y); 6 Cover type / subtype (Drop-down, mandatory Cond.: New package); 7 Package product (Drop-down, mandatory Cond.: every type except New package); 8 Reason (Drop-down, mandatory Y); 9 Comment on the reason (Text, mandatory N); 10 Negotiate with the insurers (Check box, mandatory N); 11 Market segments (Check boxes, mandatory N); 12 Heading / Details (Text, mandatory Cond.: sections or coverages before submission); 13 Coverage (Drop-down, mandatory Cond.: sections or coverages before submission); 14 Included (Check box, mandatory N); 15 Limit (Number, mandatory N); 16 Deductible (Text, mandatory N); 17 Requested rate % (Number, mandatory N); 18 Minimum premium (Number, mandatory N); 19 Commission % (Number, mandatory N); 20 Package TSI limit (Number, mandatory N); 21 Effective from (Date, mandatory N); 22 Package start (Date, mandatory N); 23 Package end (Date, mandatory Cond.: before submission (not for Retire)); 24 Anniversary (Date, mandatory N); 25 Insurer check boxes (Check boxes, mandatory Cond.: at least one when the insurers are approached); 26 Documents panel (Upload, mandatory N).
 Actions: Load Current Terms; Save Draft; Submit for Approval.
 The message of the field table is shown word for word and nothing is saved.</t>
         </is>
@@ -30542,11 +30542,11 @@
         <is>
           <t>Each message is shown word for word, with its code as the Reference for a server message, and nothing is saved:
 MSG-PM-123: "Describe the change"
-MSG-PM-128: "&lt;label&gt; already exists: &lt;key&gt;" (DUPLICATE)
-MSG-PM-129: "Complete the parameters of the &lt;type&gt; rule" (FIELD_RULE_INCOMPLETE)
-MSG-PM-130: "Unknown list of values &lt;lov type&gt;" (LOV_TYPE_UNKNOWN)
-MSG-PM-131: "&lt;label&gt; not found: &lt;id&gt;" (NOT_FOUND)
-MSG-PM-132: "Rules for every product use the scope code '*'" (RULE_SCOPE_INVALID)</t>
+MSG-PM-129: "&lt;label&gt; already exists: &lt;key&gt;" (DUPLICATE)
+MSG-PM-130: "Complete the parameters of the &lt;type&gt; rule" (FIELD_RULE_INCOMPLETE)
+MSG-PM-131: "Unknown list of values &lt;lov type&gt;" (LOV_TYPE_UNKNOWN)
+MSG-PM-132: "&lt;label&gt; not found: &lt;id&gt;" (NOT_FOUND)
+MSG-PM-133: "Rules for every product use the scope code '*'" (RULE_SCOPE_INVALID)</t>
         </is>
       </c>
       <c r="M259" s="12" t="inlineStr">
@@ -30621,29 +30621,29 @@
       <c r="L260" s="12" t="inlineStr">
         <is>
           <t>Each message is shown word for word, with its code as the Reference for a server message, and nothing is saved:
-MSG-PM-134: "Correct the highlighted fields"
-MSG-PM-135: "Enter a commission between 0 and 100"
-MSG-PM-136: "Enter a positive amount"
-MSG-PM-137: "Enter a rate between 0 and 100"
-MSG-PM-138: "Enter the effective date"
-MSG-PM-139: "Enter the minimum premium"
-MSG-PM-140: "Enter the package rate or a rate for every insurer"
-MSG-PM-141: "Include at least one coverage"
-MSG-PM-145: "The effective date cannot be before today"
-MSG-PM-146: "The package end date must be after the effective date"
-MSG-PM-147: "The package version is validated and released for use."
-MSG-PM-150: "A package version is validated by someone other than its maker and submitter" (MAKER_CHECKER_VIOLATION)
-MSG-PM-151: "Package version not found: &lt;version no&gt;" (NOT_FOUND)
-MSG-PM-152: "Enter the effective date" (PACKAGE_DATES_INVALID)
-MSG-PM-153: "The effective date cannot be before today" (PACKAGE_DATES_INVALID)
-MSG-PM-154: "The effective date must be after the start of version &lt;version no&gt;" (PACKAGE_DATES_INVALID)
-MSG-PM-155: "The package end date must be after the effective date" (PACKAGE_DATES_INVALID)
-MSG-PM-156: "The package needs its cover type and at least one included basic coverage" (PACKAGE_HIERARCHY_INCOMPLETE)
-MSG-PM-157: "Insurer &lt;insurer code&gt; has no terms for coverage &lt;coverage&gt;" (PACKAGE_INSURER_TERMS_MISSING)
-MSG-PM-158: "Enter the package rate or a rate for every insurer" (PACKAGE_RATE_MISSING)
-MSG-PM-159: "The co-insurance shares must add up to 100%" (PACKAGE_SHARES_INVALID)
-MSG-PM-160: "Enter the reason of the return" (REASON_REQUIRED)
-MSG-PM-161: "Version &lt;version no&gt; is &lt;status&gt;" (VERSION_NOT_FOR_VALIDATION)</t>
+MSG-PM-135: "Correct the highlighted fields"
+MSG-PM-136: "Enter a commission between 0 and 100"
+MSG-PM-137: "Enter a positive amount"
+MSG-PM-138: "Enter a rate between 0 and 100"
+MSG-PM-139: "Enter the effective date"
+MSG-PM-140: "Enter the minimum premium"
+MSG-PM-141: "Enter the package rate or a rate for every insurer"
+MSG-PM-142: "Include at least one coverage"
+MSG-PM-146: "The effective date cannot be before today"
+MSG-PM-147: "The package end date must be after the effective date"
+MSG-PM-148: "The package version is validated and released for use."
+MSG-PM-151: "A package version is validated by someone other than its maker and submitter" (MAKER_CHECKER_VIOLATION)
+MSG-PM-152: "Package version not found: &lt;version no&gt;" (NOT_FOUND)
+MSG-PM-153: "Enter the effective date" (PACKAGE_DATES_INVALID)
+MSG-PM-154: "The effective date cannot be before today" (PACKAGE_DATES_INVALID)
+MSG-PM-155: "The effective date must be after the start of version &lt;version no&gt;" (PACKAGE_DATES_INVALID)
+MSG-PM-156: "The package end date must be after the effective date" (PACKAGE_DATES_INVALID)
+MSG-PM-157: "The package needs its cover type and at least one included basic coverage" (PACKAGE_HIERARCHY_INCOMPLETE)
+MSG-PM-158: "Insurer &lt;insurer code&gt; has no terms for coverage &lt;coverage&gt;" (PACKAGE_INSURER_TERMS_MISSING)
+MSG-PM-159: "Enter the package rate or a rate for every insurer" (PACKAGE_RATE_MISSING)
+MSG-PM-160: "The co-insurance shares must add up to 100%" (PACKAGE_SHARES_INVALID)
+MSG-PM-161: "Enter the reason of the return" (REASON_REQUIRED)
+MSG-PM-162: "Version &lt;version no&gt; is &lt;status&gt;" (VERSION_NOT_FOR_VALIDATION)</t>
         </is>
       </c>
       <c r="M260" s="12" t="inlineStr">
@@ -30718,17 +30718,17 @@
       <c r="L261" s="12" t="inlineStr">
         <is>
           <t>Each message is shown word for word, with its code as the Reference for a server message, and nothing is saved:
-MSG-PM-164: "Enter the effective date"
-MSG-PM-165: "Enter the name"
-MSG-PM-166: "Enter the title"
-MSG-PM-167: "Enter the wording"
-MSG-PM-169: "Select the kind"
-MSG-PM-170: "Select the product line"
-MSG-PM-172: "The end is before the start"
-MSG-PM-173: "Use A-Z, 0-9 and _"
-MSG-PM-174: "&lt;label&gt; already exists: &lt;key&gt;" (DUPLICATE)
-MSG-PM-175: "&lt;label&gt; not found: &lt;code&gt;" (NOT_FOUND)
-MSG-PM-176: "&lt;label&gt; not found: &lt;id&gt;" (NOT_FOUND)</t>
+MSG-PM-165: "Enter the effective date"
+MSG-PM-166: "Enter the name"
+MSG-PM-167: "Enter the title"
+MSG-PM-168: "Enter the wording"
+MSG-PM-170: "Select the kind"
+MSG-PM-171: "Select the product line"
+MSG-PM-173: "The end is before the start"
+MSG-PM-174: "Use A-Z, 0-9 and _"
+MSG-PM-175: "&lt;label&gt; already exists: &lt;key&gt;" (DUPLICATE)
+MSG-PM-176: "&lt;label&gt; not found: &lt;code&gt;" (NOT_FOUND)
+MSG-PM-177: "&lt;label&gt; not found: &lt;id&gt;" (NOT_FOUND)</t>
         </is>
       </c>
       <c r="M261" s="12" t="inlineStr">
@@ -30803,25 +30803,25 @@
       <c r="L262" s="12" t="inlineStr">
         <is>
           <t>Each message is shown word for word, with its code as the Reference for a server message, and nothing is saved:
-MSG-PM-179: "Enter a value for each parameter"
-MSG-PM-180: "Enter the name"
-MSG-PM-181: "Enter the start date"
-MSG-PM-182: "Enter the value"
-MSG-PM-183: "Select at least one product of the matrix"
-MSG-PM-184: "Select the parameter"
-MSG-PM-185: "Select the type"
-MSG-PM-186: "The change must start after &lt;active from&gt;"
-MSG-PM-187: "The end is before the start"
-MSG-PM-188: "Use A-Z, 0-9, _ and -"
-MSG-PM-189: "An active criterion is changed by amending it (successor)" (INCENTIVE_ACTIVE_LOCKED)
-MSG-PM-190: "Only an active criterion is amended; change the pending row" (INCENTIVE_NOT_ACTIVE)
-MSG-PM-191: "The amendment must start after &lt;effective from&gt;" (INCENTIVE_PERIOD_INVALID)
-MSG-PM-192: "Criterion &lt;code&gt; already covers part of this period" (INCENTIVE_PERIOD_OVERLAP)
-MSG-PM-193: "Select at least one product of the products matrix" (INCENTIVE_PRODUCTS_REQUIRED)
-MSG-PM-194: "Product &lt;product code&gt; is not an active product of the matrix" (INCENTIVE_PRODUCT_NOT_ACTIVE)
-MSG-PM-195: "Enter the rule parameters as parameter and value rows" (INCENTIVE_RULE_PARAMS_INVALID)
-MSG-PM-196: "Enter the value of the incentive criterion" (INCENTIVE_VALUE_REQUIRED)
-MSG-PM-197: "&lt;label&gt; not found: &lt;id&gt;" (NOT_FOUND)</t>
+MSG-PM-180: "Enter a value for each parameter"
+MSG-PM-181: "Enter the name"
+MSG-PM-182: "Enter the start date"
+MSG-PM-183: "Enter the value"
+MSG-PM-184: "Select at least one product of the matrix"
+MSG-PM-185: "Select the parameter"
+MSG-PM-186: "Select the type"
+MSG-PM-187: "The change must start after &lt;active from&gt;"
+MSG-PM-188: "The end is before the start"
+MSG-PM-189: "Use A-Z, 0-9, _ and -"
+MSG-PM-190: "An active criterion is changed by amending it (successor)" (INCENTIVE_ACTIVE_LOCKED)
+MSG-PM-191: "Only an active criterion is amended; change the pending row" (INCENTIVE_NOT_ACTIVE)
+MSG-PM-192: "The amendment must start after &lt;effective from&gt;" (INCENTIVE_PERIOD_INVALID)
+MSG-PM-193: "Criterion &lt;code&gt; already covers part of this period" (INCENTIVE_PERIOD_OVERLAP)
+MSG-PM-194: "Select at least one product of the products matrix" (INCENTIVE_PRODUCTS_REQUIRED)
+MSG-PM-195: "Product &lt;product code&gt; is not an active product of the matrix" (INCENTIVE_PRODUCT_NOT_ACTIVE)
+MSG-PM-196: "Enter the rule parameters as parameter and value rows" (INCENTIVE_RULE_PARAMS_INVALID)
+MSG-PM-197: "Enter the value of the incentive criterion" (INCENTIVE_VALUE_REQUIRED)
+MSG-PM-198: "&lt;label&gt; not found: &lt;id&gt;" (NOT_FOUND)</t>
         </is>
       </c>
       <c r="M262" s="12" t="inlineStr">
@@ -30896,17 +30896,17 @@
       <c r="L263" s="12" t="inlineStr">
         <is>
           <t>Each message is shown word for word, with its code as the Reference for a server message, and nothing is saved:
-MSG-PM-200: "Default credit days must be between 0 and 365" (CREDIT_DAYS_INVALID)
-MSG-PM-201: "&lt;label&gt; already exists: &lt;key&gt;" (DUPLICATE)
-MSG-PM-202: "Branch &lt;branch code&gt; is not authorized or inactive" (INSURER_BRANCH_NOT_ACTIVE)
-MSG-PM-203: "Insurer &lt;party code&gt; has no branch &lt;branch code&gt;" (INSURER_BRANCH_UNKNOWN)
-MSG-PM-204: "Insurer &lt;party code&gt; is not authorized or is inactive" (INSURER_NOT_ACTIVE)
-MSG-PM-205: "&lt;label&gt; not found: &lt;branch id&gt;" (NOT_FOUND)
-MSG-PM-206: "&lt;label&gt; not found: &lt;id&gt;" (NOT_FOUND)
-MSG-PM-207: "&lt;label&gt; not found: &lt;party code&gt;" (NOT_FOUND)
-MSG-PM-208: "Party &lt;party code&gt; exists and is not an insurer" (PARTY_NOT_INSURER)
-MSG-PM-209: "Only e-mail placement is available; choose the e-mail placement channel" (PLACEMENT_CHANNEL_PARKED)
-MSG-PM-210: "The LGT rate must be between 0 and 100 %" (RATE_INVALID)</t>
+MSG-PM-201: "Default credit days must be between 0 and 365" (CREDIT_DAYS_INVALID)
+MSG-PM-202: "&lt;label&gt; already exists: &lt;key&gt;" (DUPLICATE)
+MSG-PM-203: "Branch &lt;branch code&gt; is not authorized or inactive" (INSURER_BRANCH_NOT_ACTIVE)
+MSG-PM-204: "Insurer &lt;party code&gt; has no branch &lt;branch code&gt;" (INSURER_BRANCH_UNKNOWN)
+MSG-PM-205: "Insurer &lt;party code&gt; is not authorized or is inactive" (INSURER_NOT_ACTIVE)
+MSG-PM-206: "&lt;label&gt; not found: &lt;branch id&gt;" (NOT_FOUND)
+MSG-PM-207: "&lt;label&gt; not found: &lt;id&gt;" (NOT_FOUND)
+MSG-PM-208: "&lt;label&gt; not found: &lt;party code&gt;" (NOT_FOUND)
+MSG-PM-209: "Party &lt;party code&gt; exists and is not an insurer" (PARTY_NOT_INSURER)
+MSG-PM-210: "Only e-mail placement is available; choose the e-mail placement channel" (PLACEMENT_CHANNEL_PARKED)
+MSG-PM-211: "The LGT rate must be between 0 and 100 %" (RATE_INVALID)</t>
         </is>
       </c>
       <c r="M263" s="12" t="inlineStr">
@@ -30981,13 +30981,13 @@
       <c r="L264" s="12" t="inlineStr">
         <is>
           <t>Each message is shown word for word, with its code as the Reference for a server message, and nothing is saved:
-MSG-PM-214: "Enter the effective-from date" (EFFECTIVE_FROM_REQUIRED)
-MSG-PM-215: "The effective-to date is before the effective-from date" (EFFECTIVITY_INVALID)
-MSG-PM-216: "The limit must be greater than zero" (LIMIT_INVALID)
-MSG-PM-217: "The premium cannot be negative" (LIMIT_PREMIUM_INVALID)
-MSG-PM-218: "&lt;label&gt; not found: &lt;id&gt;" (NOT_FOUND)
-MSG-PM-219: "&lt;label&gt; must be a percentage between 0 and 100" (RATE_INVALID)
-MSG-PM-220: "Months covered must be between 1 and 12" (SHORT_PERIOD_MONTHS_INVALID)</t>
+MSG-PM-215: "Enter the effective-from date" (EFFECTIVE_FROM_REQUIRED)
+MSG-PM-216: "The effective-to date is before the effective-from date" (EFFECTIVITY_INVALID)
+MSG-PM-217: "The limit must be greater than zero" (LIMIT_INVALID)
+MSG-PM-218: "The premium cannot be negative" (LIMIT_PREMIUM_INVALID)
+MSG-PM-219: "&lt;label&gt; not found: &lt;id&gt;" (NOT_FOUND)
+MSG-PM-220: "&lt;label&gt; must be a percentage between 0 and 100" (RATE_INVALID)
+MSG-PM-221: "Months covered must be between 1 and 12" (SHORT_PERIOD_MONTHS_INVALID)</t>
         </is>
       </c>
       <c r="M264" s="12" t="inlineStr">
@@ -31054,19 +31054,19 @@
       <c r="L265" s="12" t="inlineStr">
         <is>
           <t>Each message is shown word for word, with its code as the Reference for a server message, and nothing is saved:
-MSG-PM-228: "&lt;label&gt; already exists: &lt;key&gt;" (DUPLICATE)
-MSG-PM-229: "&lt;label&gt; not found: &lt;id&gt;" (NOT_FOUND)
-MSG-PM-230: "&lt;label&gt; not found: &lt;unit code&gt;" (NOT_FOUND)
-MSG-PM-231: "Enter the reason" (REASON_REQUIRED)
-MSG-PM-232: "&lt;&gt; is already removed from the team" (SALES_OFFICER_INACTIVE)
-MSG-PM-233: "A &lt;level&gt; must belong to an active &lt;parent level&gt;" (SALES_PARENT_INVALID)
-MSG-PM-234: "Reactivate &lt;parent code&gt; before &lt;code&gt;" (SALES_PARENT_INVALID)
-MSG-PM-235: "Team &lt;team code&gt; is unknown or inactive" (SALES_TEAM_UNKNOWN)
-MSG-PM-236: "Unit &lt;code&gt; is already inactive" (SALES_UNIT_INACTIVE)
-MSG-PM-237: "&lt;code&gt; still has &lt;open&gt;: deactivate or move them before deactivating the unit" (SALES_UNIT_IN_USE)
-MSG-PM-238: "Unit &lt;code&gt; is not inactive" (SALES_UNIT_NOT_INACTIVE)
-MSG-PM-239: "Unknown user &lt;head&gt;" (USER_UNKNOWN)
-MSG-PM-240: "Unknown user &lt;username&gt;" (USER_UNKNOWN)</t>
+MSG-PM-229: "&lt;label&gt; already exists: &lt;key&gt;" (DUPLICATE)
+MSG-PM-230: "&lt;label&gt; not found: &lt;id&gt;" (NOT_FOUND)
+MSG-PM-231: "&lt;label&gt; not found: &lt;unit code&gt;" (NOT_FOUND)
+MSG-PM-232: "Enter the reason" (REASON_REQUIRED)
+MSG-PM-233: "&lt;&gt; is already removed from the team" (SALES_OFFICER_INACTIVE)
+MSG-PM-234: "A &lt;level&gt; must belong to an active &lt;parent level&gt;" (SALES_PARENT_INVALID)
+MSG-PM-235: "Reactivate &lt;parent code&gt; before &lt;code&gt;" (SALES_PARENT_INVALID)
+MSG-PM-236: "Team &lt;team code&gt; is unknown or inactive" (SALES_TEAM_UNKNOWN)
+MSG-PM-237: "Unit &lt;code&gt; is already inactive" (SALES_UNIT_INACTIVE)
+MSG-PM-238: "&lt;code&gt; still has &lt;open&gt;: deactivate or move them before deactivating the unit" (SALES_UNIT_IN_USE)
+MSG-PM-239: "Unit &lt;code&gt; is not inactive" (SALES_UNIT_NOT_INACTIVE)
+MSG-PM-240: "Unknown user &lt;head&gt;" (USER_UNKNOWN)
+MSG-PM-241: "Unknown user &lt;username&gt;" (USER_UNKNOWN)</t>
         </is>
       </c>
       <c r="M265" s="12" t="inlineStr">
@@ -31141,18 +31141,18 @@
       <c r="L266" s="12" t="inlineStr">
         <is>
           <t>Each message is shown word for word, with its code as the Reference for a server message, and nothing is saved:
-MSG-PM-241: "Insurer &lt;insurer code&gt; is not on the panel of &lt;product code&gt; version &lt;version no&gt;" (INSURER_NOT_ON_PACKAGE)
-MSG-PM-242: "&lt;coverage&gt; limit &lt;to plain string&gt; is not in the limit table" (MOTOR_LIMIT_UNKNOWN)
-MSG-PM-243: "Package &lt;code&gt; expired and has no current version" (PRODUCT_NOT_SELLABLE)
-MSG-PM-244: "Package &lt;code&gt; has no released version in force" (PRODUCT_NOT_SELLABLE)
-MSG-PM-245: "Package &lt;code&gt; is &lt;lifecycle status&gt;: it is locked for new business" (PRODUCT_NOT_SELLABLE)
-MSG-PM-246: "Enter at least one item to rate" (RATING_NO_ITEMS)
-MSG-PM-247: "The motor OD/Theft coverage factor is not set up" (RATING_OD_FACTOR_MISSING)
-MSG-PM-248: "The period end must be after the period start" (RATING_PERIOD_INVALID)
-MSG-PM-249: "Enter the premium rate of &lt;item&gt;" (RATING_RATE_REQUIRED)
-MSG-PM-250: "No short-period percentage applies to this period" (RATING_SHORT_PERIOD_INVALID)
-MSG-PM-251: "Enter a sum insured of zero or more for every item" (RATING_SUM_INSURED_INVALID)
-MSG-PM-252: "No short-period rate is set up for &lt;months&gt; month(s)" (SHORT_PERIOD_RATE_MISSING)</t>
+MSG-PM-242: "Insurer &lt;insurer code&gt; is not on the panel of &lt;product code&gt; version &lt;version no&gt;" (INSURER_NOT_ON_PACKAGE)
+MSG-PM-243: "&lt;coverage&gt; limit &lt;to plain string&gt; is not in the limit table" (MOTOR_LIMIT_UNKNOWN)
+MSG-PM-244: "Package &lt;code&gt; expired and has no current version" (PRODUCT_NOT_SELLABLE)
+MSG-PM-245: "Package &lt;code&gt; has no released version in force" (PRODUCT_NOT_SELLABLE)
+MSG-PM-246: "Package &lt;code&gt; is &lt;lifecycle status&gt;: it is locked for new business" (PRODUCT_NOT_SELLABLE)
+MSG-PM-247: "Enter at least one item to rate" (RATING_NO_ITEMS)
+MSG-PM-248: "The motor OD/Theft coverage factor is not set up" (RATING_OD_FACTOR_MISSING)
+MSG-PM-249: "The period end must be after the period start" (RATING_PERIOD_INVALID)
+MSG-PM-250: "Enter the premium rate of &lt;item&gt;" (RATING_RATE_REQUIRED)
+MSG-PM-251: "No short-period percentage applies to this period" (RATING_SHORT_PERIOD_INVALID)
+MSG-PM-252: "Enter a sum insured of zero or more for every item" (RATING_SUM_INSURED_INVALID)
+MSG-PM-253: "No short-period rate is set up for &lt;months&gt; month(s)" (SHORT_PERIOD_RATE_MISSING)</t>
         </is>
       </c>
       <c r="M266" s="12" t="inlineStr">
@@ -31227,14 +31227,14 @@
       <c r="L267" s="12" t="inlineStr">
         <is>
           <t>Each message is shown word for word, with its code as the Reference for a server message, and nothing is saved:
-MSG-PM-254: "A rate exception is decided by someone other than its requester" (MAKER_CHECKER_VIOLATION)
-MSG-PM-255: "&lt;label&gt; not found: &lt;reference&gt;" (NOT_FOUND)
-MSG-PM-256: "Only package rate schemes need an exception" (PRODUCT_NOT_PACKAGED)
-MSG-PM-257: "Enter the version or the rate the exception is for" (RATE_EXCEPTION_INCOMPLETE)
-MSG-PM-258: "The validity date cannot be in the past" (RATE_EXCEPTION_VALIDITY_PAST)
-MSG-PM-259: "Package &lt;product code&gt; is priced on the current rate scheme: &lt;what&gt; needs an approved rate exception" (RATE_SCHEME_NOT_CURRENT)
-MSG-PM-260: "Rate exception &lt;reference&gt; does not approve &lt;what&gt; for &lt;product code&gt;" (RATE_SCHEME_NOT_CURRENT)
-MSG-PM-261: "Rate exception &lt;reference no&gt; is already decided" (RECORD_NOT_PENDING)</t>
+MSG-PM-255: "A rate exception is decided by someone other than its requester" (MAKER_CHECKER_VIOLATION)
+MSG-PM-256: "&lt;label&gt; not found: &lt;reference&gt;" (NOT_FOUND)
+MSG-PM-257: "Only package rate schemes need an exception" (PRODUCT_NOT_PACKAGED)
+MSG-PM-258: "Enter the version or the rate the exception is for" (RATE_EXCEPTION_INCOMPLETE)
+MSG-PM-259: "The validity date cannot be in the past" (RATE_EXCEPTION_VALIDITY_PAST)
+MSG-PM-260: "Package &lt;product code&gt; is priced on the current rate scheme: &lt;what&gt; needs an approved rate exception" (RATE_SCHEME_NOT_CURRENT)
+MSG-PM-261: "Rate exception &lt;reference&gt; does not approve &lt;what&gt; for &lt;product code&gt;" (RATE_SCHEME_NOT_CURRENT)
+MSG-PM-262: "Rate exception &lt;reference no&gt; is already decided" (RECORD_NOT_PENDING)</t>
         </is>
       </c>
       <c r="M267" s="12" t="inlineStr">
@@ -31297,7 +31297,7 @@
       <c r="L268" s="12" t="inlineStr">
         <is>
           <t>Each message is shown word for word, with its code as the Reference for a server message, and nothing is saved:
-MSG-PM-262: "&lt;label&gt; not found: &lt;id&gt;" (NOT_FOUND)</t>
+MSG-PM-263: "&lt;label&gt; not found: &lt;id&gt;" (NOT_FOUND)</t>
         </is>
       </c>
       <c r="M268" s="12" t="inlineStr">
@@ -31360,13 +31360,13 @@
       <c r="L269" s="12" t="inlineStr">
         <is>
           <t>Each message is shown word for word, with its code as the Reference for a server message, and nothing is saved:
-MSG-PM-263: "You are not permitted to perform this action" (ACCESS_DENIED)
-MSG-PM-264: "The record was changed by another user. Please reload and try again." (CONCURRENT_MODIFICATION)
-MSG-PM-266: "The system could not complete the request. Try again; if it continues, contact support with the reference." (INTERNAL_ERROR)
-MSG-PM-268: "Parameter '&lt;name&gt;' has an invalid value" (MALFORMED_REQUEST)
-MSG-PM-269: "Required parameter '&lt;parameter name&gt;' is missing" (MALFORMED_REQUEST)
-MSG-PM-274: "The uploaded file is too large" (UPLOAD_TOO_LARGE)
-MSG-PM-275: "Invalid request" (VALIDATION_FAILED)</t>
+MSG-PM-264: "You are not permitted to perform this action" (ACCESS_DENIED)
+MSG-PM-265: "The record was changed by another user. Please reload and try again." (CONCURRENT_MODIFICATION)
+MSG-PM-267: "The system could not complete the request. Try again; if it continues, contact support with the reference." (INTERNAL_ERROR)
+MSG-PM-269: "Parameter '&lt;name&gt;' has an invalid value" (MALFORMED_REQUEST)
+MSG-PM-270: "Required parameter '&lt;parameter name&gt;' is missing" (MALFORMED_REQUEST)
+MSG-PM-275: "The uploaded file is too large" (UPLOAD_TOO_LARGE)
+MSG-PM-276: "Invalid request" (VALIDATION_FAILED)</t>
         </is>
       </c>
       <c r="M269" s="12" t="inlineStr">
@@ -31429,12 +31429,12 @@
       <c r="L270" s="12" t="inlineStr">
         <is>
           <t>Each message is shown word for word, with its code as the Reference for a server message, and nothing is saved:
-MSG-PM-265: "&lt;label&gt; already exists: &lt;key&gt;" (DUPLICATE)
-MSG-PM-267: "A rate exception is decided by someone other than its requester" (MAKER_CHECKER_VIOLATION)
-MSG-PM-270: "&lt;label&gt; not found: &lt;id&gt;" (NOT_FOUND)
-MSG-PM-271: "Product &lt;code&gt; was not created by the migration" (PRODUCT_NOT_MIGRATED)
-MSG-PM-272: "Enter the reason for the rejection" (RATE_EXCEPTION_REASON_REQUIRED)
-MSG-PM-273: "Rate exception &lt;reference&gt; is already decided" (RECORD_NOT_PENDING)</t>
+MSG-PM-266: "&lt;label&gt; already exists: &lt;key&gt;" (DUPLICATE)
+MSG-PM-268: "A rate exception is decided by someone other than its requester" (MAKER_CHECKER_VIOLATION)
+MSG-PM-271: "&lt;label&gt; not found: &lt;id&gt;" (NOT_FOUND)
+MSG-PM-272: "Product &lt;code&gt; was not created by the migration" (PRODUCT_NOT_MIGRATED)
+MSG-PM-273: "Enter the reason for the rejection" (RATE_EXCEPTION_REASON_REQUIRED)
+MSG-PM-274: "Rate exception &lt;reference&gt; is already decided" (RECORD_NOT_PENDING)</t>
         </is>
       </c>
       <c r="M270" s="12" t="inlineStr">

</xml_diff>

<commit_message>
Client documents in the new wording: BIBS in the BRD-11 e-mails and sign-in, BRD-05 close date and time fields and tax message, CPC2 without the seed marker in BRD-01 and BRD-03 cases, BRD-13 error rate 0.00%; rebuilt BRD-01, BRD-03, BRD-13 04, BRD-11 02 and 03, BRD-13 02
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01W3DAuLtsQmip7EuxjJCCtN
</commit_message>
<xml_diff>
--- a/docs/deliverables/out/Drop-0_Setup_and_Data_Migration/BRD-03_Product_Maintenance/04_BIBS_TestPlan_BRD-03_Product_Maintenance_v2.0.xlsx
+++ b/docs/deliverables/out/Drop-0_Setup_and_Data_Migration/BRD-03_Product_Maintenance/04_BIBS_TestPlan_BRD-03_Product_Maintenance_v2.0.xlsx
@@ -26915,7 +26915,7 @@
       </c>
       <c r="K213" s="12" t="inlineStr">
         <is>
-          <t>1. Click New Criterion; code UAT1, name "UAT campaign", type Sales campaign (seed), value basis Fixed amount, value 500, effective from today; products MTR12; save.
+          <t>1. Click New Criterion; code UAT1, name "UAT campaign", type Sales campaign, value basis Fixed amount, value 500, effective from today; products MTR12; save.
 2. As badmin authorise it in My Approvals.</t>
         </is>
       </c>
@@ -28369,7 +28369,7 @@
       <c r="L232" s="12" t="inlineStr">
         <is>
           <t>The screen matches SCR-PM-05 Package Request record: Negotiation tab of the FRS.
-Fields in this order: 1 Round n · slip number (Card title, mandatory -); 2 Round status pill and Locked tag (Pill, mandatory -); 3 Round note (Text, mandatory -); 4 Insurer check boxes (Check boxes, mandatory Y (at least one)); 5 Notes to the insurers (Text, mandatory N); 6 Insurer (Column, mandatory -); 7 Outcome (Column, mandatory -); 8 Rate % / Minimum / Conditions / Valid Until (Column, mandatory -); 9 Rev. (Column, mandatory -); 10 Outcome (Drop-down, mandatory Y); 11 Rate % (Number, mandatory Cond.: an offer (accepted, approved with changes, counter-proposal)); 12 Minimum premium (Number, mandatory N); 13 Valid until (Date, mandatory N); 14 Deductible per coverage (Text, mandatory N); 15 Conditions and warranties (Text, mandatory N); 16 Remarks (Text, mandatory N); 17 Response document (File, mandatory N); 18 Offer check box (Check box, mandatory Y (at least one)); 19 Role (Drop-down, mandatory Y); 20 Share % (Number, mandatory Cond.: co-insurance (lead and participants)); 21 Comment (Text, mandatory N); 22 Insurer check boxes (Check boxes, mandatory Y (at least one)); 23 What changes in this round (Text, mandatory N).
+Fields in this order: 1 Round n · slip number (Card title, mandatory -); 2 Round status pill and Locked tag (Pill, mandatory -); 3 Round note (Text, mandatory -); 4 Insurer check boxes (Check boxes, mandatory Y (at least one)); 5 Notes to the insurers (Text, mandatory N); 6 Insurer (Column, mandatory -); 7 Outcome (Column, mandatory -); 8 Rate % / Minimum / Conditions / Valid Until (Column, mandatory -); 9 Rev. (Column, mandatory -); 10 Row action menu (Row action menu, mandatory -); 11 Outcome (Drop-down, mandatory Y); 12 Rate % (Number, mandatory Cond.: an offer (accepted, approved with changes, counter-proposal)); 13 Minimum premium (Number, mandatory N); 14 Valid until (Date, mandatory N); 15 Deductible per coverage (Text, mandatory N); 16 Conditions and warranties (Text, mandatory N); 17 Remarks (Text, mandatory N); 18 Response document (File, mandatory N); 19 Offer check box (Check box, mandatory Y (at least one)); 20 Role (Drop-down, mandatory Y); 21 Share % (Number, mandatory Cond.: co-insurance (lead and participants)); 22 Comment (Text, mandatory N); 23 Insurer check boxes (Check boxes, mandatory Y (at least one)); 24 What changes in this round (Text, mandatory N).
 Actions: Save Slip; Submit for Approval; Approve and Send; Quotation Slip; Key In; Save Terms; Resend; Revise quotation slip (new round); Terms final.
 The message of the field table is shown word for word and nothing is saved.</t>
         </is>
@@ -35148,7 +35148,7 @@
       </c>
       <c r="C13" s="12" t="inlineStr">
         <is>
-          <t>CPC2 (seed), type CAMPAIGN, value basis RATE 1.00, on Motor and Property packages, ACTIVE</t>
+          <t>CPC2, type CAMPAIGN, value basis RATE 1.00, on Motor and Property packages, ACTIVE</t>
         </is>
       </c>
       <c r="D13" s="12" t="inlineStr">

</xml_diff>